<commit_message>
further tests and development of defoliation #104
</commit_message>
<xml_diff>
--- a/data-raw/data_input_defoliation.xlsx
+++ b/data-raw/data_input_defoliation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trotsiuk/Documents/Research/software/r3PG/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{188C1FD1-F10D-A740-BA95-24B996E35CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF43C66-D51C-614A-BC71-E09B5D04E354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33140" yWindow="500" windowWidth="43660" windowHeight="31500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10160" yWindow="500" windowWidth="43660" windowHeight="31500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="site" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="162">
   <si>
     <t>latitude</t>
   </si>
@@ -523,6 +523,9 @@
   <si>
     <t>prop_npp</t>
   </si>
+  <si>
+    <t>def_type</t>
+  </si>
 </sst>
 </file>
 
@@ -25061,10 +25064,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A88D5E7-4ED0-6C46-95F2-C0683DE408CB}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -25072,28 +25075,31 @@
         <v>25</v>
       </c>
       <c r="C1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D1" t="s">
         <v>155</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>156</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>157</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>26</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>158</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>159</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>153</v>
       </c>
@@ -25101,24 +25107,27 @@
         <v>70</v>
       </c>
       <c r="C2">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="D2">
         <v>0.5</v>
       </c>
       <c r="E2">
+        <v>0.5</v>
+      </c>
+      <c r="F2">
         <v>0.1</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G2" s="2">
         <v>1</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>60</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>0.4</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>0.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Removed error (and unrealistic thinning stems_n) in "defoliation" and "thinning" inputs in: data-raw/data_input_defoliation.xlsx
</commit_message>
<xml_diff>
--- a/data-raw/data_input_defoliation.xlsx
+++ b/data-raw/data_input_defoliation.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\thinning_defoliation_events\Rdata\data\revised_files_Vova\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Forrester\Models\3-PG\r3PG_mortality_management_defoliation\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C5B5D91-A7C7-4A78-BF07-A3B545FB9A23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC239BB-073A-4A17-87CE-78ECD6F6FB86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="site" sheetId="1" r:id="rId1"/>
@@ -25083,7 +25083,7 @@
         <v>60</v>
       </c>
       <c r="C2">
-        <v>0.5</v>
+        <v>100</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -25157,10 +25157,10 @@
         <v>0.5</v>
       </c>
       <c r="E2">
+        <v>0.6</v>
+      </c>
+      <c r="F2">
         <v>0.5</v>
-      </c>
-      <c r="F2">
-        <v>0.1</v>
       </c>
       <c r="G2" s="1">
         <v>1</v>

</xml_diff>